<commit_message>
docs: add comprehensive README.md and complete stateful row delta engine
</commit_message>
<xml_diff>
--- a/data/input/test.xlsx
+++ b/data/input/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VSCode\Java\dataflow-connectors\file-connector\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5157A72D-F6DC-4BDB-B5E8-1E9FDE73683D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C137361-DE72-4612-96D1-C5E8135B931F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="9960" tabRatio="205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3384" yWindow="3384" windowWidth="17280" windowHeight="9960" tabRatio="205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -127,9 +127,6 @@
     <t>k</t>
   </si>
   <si>
-    <t>yooooo</t>
-  </si>
-  <si>
     <t>yooo</t>
   </si>
   <si>
@@ -137,6 +134,9 @@
   </si>
   <si>
     <t>12-02-1234</t>
+  </si>
+  <si>
+    <t>test101</t>
   </si>
 </sst>
 </file>
@@ -772,22 +772,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
         <v>35</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>36</v>
       </c>
-      <c r="D13" t="s">
-        <v>37</v>
-      </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F13">
         <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H13">
         <v>2523</v>

</xml_diff>